<commit_message>
update on test cases
</commit_message>
<xml_diff>
--- a/documents/ParaBank_Test_Cases.xlsx
+++ b/documents/ParaBank_Test_Cases.xlsx
@@ -3,9 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{053F5D90-1E26-40B8-900C-4778B7E8A75A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DVDSTORE\Desktop\Rawad files\My Own Files\project\qa-project\bank.system\documents\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61B8C63C-2919-4380-BD75-931C1C61FF2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-384000" yWindow="-384000" windowWidth="2388" windowHeight="564" tabRatio="500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Homepage" sheetId="1" r:id="rId1"/>
@@ -37,7 +42,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Services!$A$1:$I$8</definedName>
   </definedNames>
   <calcPr calcId="0" iterateDelta="1E-4"/>
-  <oleSize ref="A1:E4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>

</xml_diff>